<commit_message>
Improve classroom menu, rewards, opening, and student import
</commit_message>
<xml_diff>
--- a/assets/templates/student-registration-template.xlsx
+++ b/assets/templates/student-registration-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="학생등록" sheetId="1" r:id="Rbc0c0305657147df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="학생등록" sheetId="1" r:id="Re1ffe6f4c9ed405d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,9 +13,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="0"/>
-  </x:numFmts>
   <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
@@ -23,17 +20,17 @@
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="11"/>
+      <x:sz val="12"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Arial"/>
+      <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF172D37"/>
-      <x:name val="Arial"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -45,23 +42,14 @@
         <x:fgColor rgb="FF23434B"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFCF6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
-    <x:border>
-      <x:left style="thin">
-        <x:color rgb="FFFFFFFF"/>
-      </x:left>
-      <x:right style="thin">
-        <x:color rgb="FFFFFFFF"/>
-      </x:right>
-      <x:top style="thin">
-        <x:color rgb="FFFFFFFF"/>
-      </x:top>
-      <x:bottom style="thin">
-        <x:color rgb="FFFFFFFF"/>
-      </x:bottom>
-    </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD6C9B1"/>
@@ -76,11 +64,25 @@
         <x:color rgb="FFD6C9B1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE2D9C8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE2D9C8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE2D9C8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE2D9C8"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -91,29 +93,13 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -316,645 +302,634 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetPr>
-    <x:tabColor rgb="FF23434B"/>
-  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="10" t="str">
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>학년</x:v>
       </x:c>
-      <x:c r="B1" s="10" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>반</x:v>
       </x:c>
-      <x:c r="C1" s="10" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>번호</x:v>
       </x:c>
-      <x:c r="D1" s="10" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>이름</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="13" t="n">
+      <x:c r="A2" s="10" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="13" t="n">
+      <x:c r="B2" s="10" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C2" s="13" t="n">
+      <x:c r="C2" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D2" s="12" t="str">
-        <x:v>홍길동</x:v>
+      <x:c r="D2" s="9" t="str">
+        <x:v>예시_홍길동(이 행을 지우고 입력)</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="13" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="13" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="13" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="str">
-        <x:v>김철수</x:v>
-      </x:c>
+      <x:c r="A3" s="10"/>
+      <x:c r="B3" s="10"/>
+      <x:c r="C3" s="10"/>
+      <x:c r="D3" s="9"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="14"/>
-      <x:c r="B4" s="14"/>
-      <x:c r="C4" s="14"/>
+      <x:c r="A4" s="10"/>
+      <x:c r="B4" s="10"/>
+      <x:c r="C4" s="10"/>
       <x:c r="D4" s="9"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="14"/>
-      <x:c r="B5" s="14"/>
-      <x:c r="C5" s="14"/>
+      <x:c r="A5" s="10"/>
+      <x:c r="B5" s="10"/>
+      <x:c r="C5" s="10"/>
       <x:c r="D5" s="9"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="14"/>
-      <x:c r="B6" s="14"/>
-      <x:c r="C6" s="14"/>
+      <x:c r="A6" s="10"/>
+      <x:c r="B6" s="10"/>
+      <x:c r="C6" s="10"/>
       <x:c r="D6" s="9"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="14"/>
-      <x:c r="B7" s="14"/>
-      <x:c r="C7" s="14"/>
+      <x:c r="A7" s="10"/>
+      <x:c r="B7" s="10"/>
+      <x:c r="C7" s="10"/>
       <x:c r="D7" s="9"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="14"/>
-      <x:c r="B8" s="14"/>
-      <x:c r="C8" s="14"/>
+      <x:c r="A8" s="10"/>
+      <x:c r="B8" s="10"/>
+      <x:c r="C8" s="10"/>
       <x:c r="D8" s="9"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="14"/>
-      <x:c r="B9" s="14"/>
-      <x:c r="C9" s="14"/>
+      <x:c r="A9" s="10"/>
+      <x:c r="B9" s="10"/>
+      <x:c r="C9" s="10"/>
       <x:c r="D9" s="9"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="14"/>
-      <x:c r="B10" s="14"/>
-      <x:c r="C10" s="14"/>
+      <x:c r="A10" s="10"/>
+      <x:c r="B10" s="10"/>
+      <x:c r="C10" s="10"/>
       <x:c r="D10" s="9"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="14"/>
-      <x:c r="B11" s="14"/>
-      <x:c r="C11" s="14"/>
+      <x:c r="A11" s="10"/>
+      <x:c r="B11" s="10"/>
+      <x:c r="C11" s="10"/>
       <x:c r="D11" s="9"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="14"/>
-      <x:c r="B12" s="14"/>
-      <x:c r="C12" s="14"/>
+      <x:c r="A12" s="10"/>
+      <x:c r="B12" s="10"/>
+      <x:c r="C12" s="10"/>
       <x:c r="D12" s="9"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="14"/>
-      <x:c r="B13" s="14"/>
-      <x:c r="C13" s="14"/>
+      <x:c r="A13" s="10"/>
+      <x:c r="B13" s="10"/>
+      <x:c r="C13" s="10"/>
       <x:c r="D13" s="9"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="14"/>
-      <x:c r="B14" s="14"/>
-      <x:c r="C14" s="14"/>
+      <x:c r="A14" s="10"/>
+      <x:c r="B14" s="10"/>
+      <x:c r="C14" s="10"/>
       <x:c r="D14" s="9"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="14"/>
-      <x:c r="B15" s="14"/>
-      <x:c r="C15" s="14"/>
+      <x:c r="A15" s="10"/>
+      <x:c r="B15" s="10"/>
+      <x:c r="C15" s="10"/>
       <x:c r="D15" s="9"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="14"/>
-      <x:c r="B16" s="14"/>
-      <x:c r="C16" s="14"/>
+      <x:c r="A16" s="10"/>
+      <x:c r="B16" s="10"/>
+      <x:c r="C16" s="10"/>
       <x:c r="D16" s="9"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="14"/>
-      <x:c r="B17" s="14"/>
-      <x:c r="C17" s="14"/>
+      <x:c r="A17" s="10"/>
+      <x:c r="B17" s="10"/>
+      <x:c r="C17" s="10"/>
       <x:c r="D17" s="9"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="14"/>
-      <x:c r="B18" s="14"/>
-      <x:c r="C18" s="14"/>
+      <x:c r="A18" s="10"/>
+      <x:c r="B18" s="10"/>
+      <x:c r="C18" s="10"/>
       <x:c r="D18" s="9"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="14"/>
-      <x:c r="C19" s="14"/>
+      <x:c r="A19" s="10"/>
+      <x:c r="B19" s="10"/>
+      <x:c r="C19" s="10"/>
       <x:c r="D19" s="9"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="14"/>
-      <x:c r="C20" s="14"/>
+      <x:c r="A20" s="10"/>
+      <x:c r="B20" s="10"/>
+      <x:c r="C20" s="10"/>
       <x:c r="D20" s="9"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="14"/>
-      <x:c r="B21" s="14"/>
-      <x:c r="C21" s="14"/>
+      <x:c r="A21" s="10"/>
+      <x:c r="B21" s="10"/>
+      <x:c r="C21" s="10"/>
       <x:c r="D21" s="9"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="14"/>
-      <x:c r="B22" s="14"/>
-      <x:c r="C22" s="14"/>
+      <x:c r="A22" s="10"/>
+      <x:c r="B22" s="10"/>
+      <x:c r="C22" s="10"/>
       <x:c r="D22" s="9"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="14"/>
-      <x:c r="B23" s="14"/>
-      <x:c r="C23" s="14"/>
+      <x:c r="A23" s="10"/>
+      <x:c r="B23" s="10"/>
+      <x:c r="C23" s="10"/>
       <x:c r="D23" s="9"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="14"/>
-      <x:c r="B24" s="14"/>
-      <x:c r="C24" s="14"/>
+      <x:c r="A24" s="10"/>
+      <x:c r="B24" s="10"/>
+      <x:c r="C24" s="10"/>
       <x:c r="D24" s="9"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="14"/>
-      <x:c r="B25" s="14"/>
-      <x:c r="C25" s="14"/>
+      <x:c r="A25" s="10"/>
+      <x:c r="B25" s="10"/>
+      <x:c r="C25" s="10"/>
       <x:c r="D25" s="9"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="14"/>
-      <x:c r="B26" s="14"/>
-      <x:c r="C26" s="14"/>
+      <x:c r="A26" s="10"/>
+      <x:c r="B26" s="10"/>
+      <x:c r="C26" s="10"/>
       <x:c r="D26" s="9"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="14"/>
-      <x:c r="B27" s="14"/>
-      <x:c r="C27" s="14"/>
+      <x:c r="A27" s="10"/>
+      <x:c r="B27" s="10"/>
+      <x:c r="C27" s="10"/>
       <x:c r="D27" s="9"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="14"/>
-      <x:c r="B28" s="14"/>
-      <x:c r="C28" s="14"/>
+      <x:c r="A28" s="10"/>
+      <x:c r="B28" s="10"/>
+      <x:c r="C28" s="10"/>
       <x:c r="D28" s="9"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="14"/>
-      <x:c r="B29" s="14"/>
-      <x:c r="C29" s="14"/>
+      <x:c r="A29" s="10"/>
+      <x:c r="B29" s="10"/>
+      <x:c r="C29" s="10"/>
       <x:c r="D29" s="9"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="14"/>
-      <x:c r="B30" s="14"/>
-      <x:c r="C30" s="14"/>
+      <x:c r="A30" s="10"/>
+      <x:c r="B30" s="10"/>
+      <x:c r="C30" s="10"/>
       <x:c r="D30" s="9"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="14"/>
-      <x:c r="B31" s="14"/>
-      <x:c r="C31" s="14"/>
+      <x:c r="A31" s="10"/>
+      <x:c r="B31" s="10"/>
+      <x:c r="C31" s="10"/>
       <x:c r="D31" s="9"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="14"/>
-      <x:c r="B32" s="14"/>
-      <x:c r="C32" s="14"/>
+      <x:c r="A32" s="10"/>
+      <x:c r="B32" s="10"/>
+      <x:c r="C32" s="10"/>
       <x:c r="D32" s="9"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="14"/>
-      <x:c r="B33" s="14"/>
-      <x:c r="C33" s="14"/>
+      <x:c r="A33" s="10"/>
+      <x:c r="B33" s="10"/>
+      <x:c r="C33" s="10"/>
       <x:c r="D33" s="9"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="14"/>
-      <x:c r="B34" s="14"/>
-      <x:c r="C34" s="14"/>
+      <x:c r="A34" s="10"/>
+      <x:c r="B34" s="10"/>
+      <x:c r="C34" s="10"/>
       <x:c r="D34" s="9"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="14"/>
-      <x:c r="B35" s="14"/>
-      <x:c r="C35" s="14"/>
+      <x:c r="A35" s="10"/>
+      <x:c r="B35" s="10"/>
+      <x:c r="C35" s="10"/>
       <x:c r="D35" s="9"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="14"/>
-      <x:c r="B36" s="14"/>
-      <x:c r="C36" s="14"/>
+      <x:c r="A36" s="10"/>
+      <x:c r="B36" s="10"/>
+      <x:c r="C36" s="10"/>
       <x:c r="D36" s="9"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="14"/>
-      <x:c r="B37" s="14"/>
-      <x:c r="C37" s="14"/>
+      <x:c r="A37" s="10"/>
+      <x:c r="B37" s="10"/>
+      <x:c r="C37" s="10"/>
       <x:c r="D37" s="9"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="14"/>
-      <x:c r="B38" s="14"/>
-      <x:c r="C38" s="14"/>
+      <x:c r="A38" s="10"/>
+      <x:c r="B38" s="10"/>
+      <x:c r="C38" s="10"/>
       <x:c r="D38" s="9"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="14"/>
-      <x:c r="B39" s="14"/>
-      <x:c r="C39" s="14"/>
+      <x:c r="A39" s="10"/>
+      <x:c r="B39" s="10"/>
+      <x:c r="C39" s="10"/>
       <x:c r="D39" s="9"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="14"/>
-      <x:c r="B40" s="14"/>
-      <x:c r="C40" s="14"/>
+      <x:c r="A40" s="10"/>
+      <x:c r="B40" s="10"/>
+      <x:c r="C40" s="10"/>
       <x:c r="D40" s="9"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="14"/>
-      <x:c r="B41" s="14"/>
-      <x:c r="C41" s="14"/>
+      <x:c r="A41" s="10"/>
+      <x:c r="B41" s="10"/>
+      <x:c r="C41" s="10"/>
       <x:c r="D41" s="9"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="14"/>
-      <x:c r="B42" s="14"/>
-      <x:c r="C42" s="14"/>
+      <x:c r="A42" s="10"/>
+      <x:c r="B42" s="10"/>
+      <x:c r="C42" s="10"/>
       <x:c r="D42" s="9"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="14"/>
-      <x:c r="B43" s="14"/>
-      <x:c r="C43" s="14"/>
+      <x:c r="A43" s="10"/>
+      <x:c r="B43" s="10"/>
+      <x:c r="C43" s="10"/>
       <x:c r="D43" s="9"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="14"/>
-      <x:c r="B44" s="14"/>
-      <x:c r="C44" s="14"/>
+      <x:c r="A44" s="10"/>
+      <x:c r="B44" s="10"/>
+      <x:c r="C44" s="10"/>
       <x:c r="D44" s="9"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="14"/>
-      <x:c r="B45" s="14"/>
-      <x:c r="C45" s="14"/>
+      <x:c r="A45" s="10"/>
+      <x:c r="B45" s="10"/>
+      <x:c r="C45" s="10"/>
       <x:c r="D45" s="9"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="14"/>
-      <x:c r="B46" s="14"/>
-      <x:c r="C46" s="14"/>
+      <x:c r="A46" s="10"/>
+      <x:c r="B46" s="10"/>
+      <x:c r="C46" s="10"/>
       <x:c r="D46" s="9"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="14"/>
-      <x:c r="B47" s="14"/>
-      <x:c r="C47" s="14"/>
+      <x:c r="A47" s="10"/>
+      <x:c r="B47" s="10"/>
+      <x:c r="C47" s="10"/>
       <x:c r="D47" s="9"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="14"/>
-      <x:c r="B48" s="14"/>
-      <x:c r="C48" s="14"/>
+      <x:c r="A48" s="10"/>
+      <x:c r="B48" s="10"/>
+      <x:c r="C48" s="10"/>
       <x:c r="D48" s="9"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="14"/>
-      <x:c r="B49" s="14"/>
-      <x:c r="C49" s="14"/>
+      <x:c r="A49" s="10"/>
+      <x:c r="B49" s="10"/>
+      <x:c r="C49" s="10"/>
       <x:c r="D49" s="9"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="14"/>
-      <x:c r="B50" s="14"/>
-      <x:c r="C50" s="14"/>
+      <x:c r="A50" s="10"/>
+      <x:c r="B50" s="10"/>
+      <x:c r="C50" s="10"/>
       <x:c r="D50" s="9"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="14"/>
-      <x:c r="B51" s="14"/>
-      <x:c r="C51" s="14"/>
+      <x:c r="A51" s="10"/>
+      <x:c r="B51" s="10"/>
+      <x:c r="C51" s="10"/>
       <x:c r="D51" s="9"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="14"/>
-      <x:c r="B52" s="14"/>
-      <x:c r="C52" s="14"/>
+      <x:c r="A52" s="10"/>
+      <x:c r="B52" s="10"/>
+      <x:c r="C52" s="10"/>
       <x:c r="D52" s="9"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="14"/>
-      <x:c r="B53" s="14"/>
-      <x:c r="C53" s="14"/>
+      <x:c r="A53" s="10"/>
+      <x:c r="B53" s="10"/>
+      <x:c r="C53" s="10"/>
       <x:c r="D53" s="9"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="14"/>
-      <x:c r="B54" s="14"/>
-      <x:c r="C54" s="14"/>
+      <x:c r="A54" s="10"/>
+      <x:c r="B54" s="10"/>
+      <x:c r="C54" s="10"/>
       <x:c r="D54" s="9"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="14"/>
-      <x:c r="B55" s="14"/>
-      <x:c r="C55" s="14"/>
+      <x:c r="A55" s="10"/>
+      <x:c r="B55" s="10"/>
+      <x:c r="C55" s="10"/>
       <x:c r="D55" s="9"/>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="14"/>
-      <x:c r="B56" s="14"/>
-      <x:c r="C56" s="14"/>
+      <x:c r="A56" s="10"/>
+      <x:c r="B56" s="10"/>
+      <x:c r="C56" s="10"/>
       <x:c r="D56" s="9"/>
     </x:row>
     <x:row r="57">
-      <x:c r="A57" s="14"/>
-      <x:c r="B57" s="14"/>
-      <x:c r="C57" s="14"/>
+      <x:c r="A57" s="10"/>
+      <x:c r="B57" s="10"/>
+      <x:c r="C57" s="10"/>
       <x:c r="D57" s="9"/>
     </x:row>
     <x:row r="58">
-      <x:c r="A58" s="14"/>
-      <x:c r="B58" s="14"/>
-      <x:c r="C58" s="14"/>
+      <x:c r="A58" s="10"/>
+      <x:c r="B58" s="10"/>
+      <x:c r="C58" s="10"/>
       <x:c r="D58" s="9"/>
     </x:row>
     <x:row r="59">
-      <x:c r="A59" s="14"/>
-      <x:c r="B59" s="14"/>
-      <x:c r="C59" s="14"/>
+      <x:c r="A59" s="10"/>
+      <x:c r="B59" s="10"/>
+      <x:c r="C59" s="10"/>
       <x:c r="D59" s="9"/>
     </x:row>
     <x:row r="60">
-      <x:c r="A60" s="14"/>
-      <x:c r="B60" s="14"/>
-      <x:c r="C60" s="14"/>
+      <x:c r="A60" s="10"/>
+      <x:c r="B60" s="10"/>
+      <x:c r="C60" s="10"/>
       <x:c r="D60" s="9"/>
     </x:row>
     <x:row r="61">
-      <x:c r="A61" s="14"/>
-      <x:c r="B61" s="14"/>
-      <x:c r="C61" s="14"/>
+      <x:c r="A61" s="10"/>
+      <x:c r="B61" s="10"/>
+      <x:c r="C61" s="10"/>
       <x:c r="D61" s="9"/>
     </x:row>
     <x:row r="62">
-      <x:c r="A62" s="14"/>
-      <x:c r="B62" s="14"/>
-      <x:c r="C62" s="14"/>
+      <x:c r="A62" s="10"/>
+      <x:c r="B62" s="10"/>
+      <x:c r="C62" s="10"/>
       <x:c r="D62" s="9"/>
     </x:row>
     <x:row r="63">
-      <x:c r="A63" s="14"/>
-      <x:c r="B63" s="14"/>
-      <x:c r="C63" s="14"/>
+      <x:c r="A63" s="10"/>
+      <x:c r="B63" s="10"/>
+      <x:c r="C63" s="10"/>
       <x:c r="D63" s="9"/>
     </x:row>
     <x:row r="64">
-      <x:c r="A64" s="14"/>
-      <x:c r="B64" s="14"/>
-      <x:c r="C64" s="14"/>
+      <x:c r="A64" s="10"/>
+      <x:c r="B64" s="10"/>
+      <x:c r="C64" s="10"/>
       <x:c r="D64" s="9"/>
     </x:row>
     <x:row r="65">
-      <x:c r="A65" s="14"/>
-      <x:c r="B65" s="14"/>
-      <x:c r="C65" s="14"/>
+      <x:c r="A65" s="10"/>
+      <x:c r="B65" s="10"/>
+      <x:c r="C65" s="10"/>
       <x:c r="D65" s="9"/>
     </x:row>
     <x:row r="66">
-      <x:c r="A66" s="14"/>
-      <x:c r="B66" s="14"/>
-      <x:c r="C66" s="14"/>
+      <x:c r="A66" s="10"/>
+      <x:c r="B66" s="10"/>
+      <x:c r="C66" s="10"/>
       <x:c r="D66" s="9"/>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="14"/>
-      <x:c r="B67" s="14"/>
-      <x:c r="C67" s="14"/>
+      <x:c r="A67" s="10"/>
+      <x:c r="B67" s="10"/>
+      <x:c r="C67" s="10"/>
       <x:c r="D67" s="9"/>
     </x:row>
     <x:row r="68">
-      <x:c r="A68" s="14"/>
-      <x:c r="B68" s="14"/>
-      <x:c r="C68" s="14"/>
+      <x:c r="A68" s="10"/>
+      <x:c r="B68" s="10"/>
+      <x:c r="C68" s="10"/>
       <x:c r="D68" s="9"/>
     </x:row>
     <x:row r="69">
-      <x:c r="A69" s="14"/>
-      <x:c r="B69" s="14"/>
-      <x:c r="C69" s="14"/>
+      <x:c r="A69" s="10"/>
+      <x:c r="B69" s="10"/>
+      <x:c r="C69" s="10"/>
       <x:c r="D69" s="9"/>
     </x:row>
     <x:row r="70">
-      <x:c r="A70" s="14"/>
-      <x:c r="B70" s="14"/>
-      <x:c r="C70" s="14"/>
+      <x:c r="A70" s="10"/>
+      <x:c r="B70" s="10"/>
+      <x:c r="C70" s="10"/>
       <x:c r="D70" s="9"/>
     </x:row>
     <x:row r="71">
-      <x:c r="A71" s="14"/>
-      <x:c r="B71" s="14"/>
-      <x:c r="C71" s="14"/>
+      <x:c r="A71" s="10"/>
+      <x:c r="B71" s="10"/>
+      <x:c r="C71" s="10"/>
       <x:c r="D71" s="9"/>
     </x:row>
     <x:row r="72">
-      <x:c r="A72" s="14"/>
-      <x:c r="B72" s="14"/>
-      <x:c r="C72" s="14"/>
+      <x:c r="A72" s="10"/>
+      <x:c r="B72" s="10"/>
+      <x:c r="C72" s="10"/>
       <x:c r="D72" s="9"/>
     </x:row>
     <x:row r="73">
-      <x:c r="A73" s="14"/>
-      <x:c r="B73" s="14"/>
-      <x:c r="C73" s="14"/>
+      <x:c r="A73" s="10"/>
+      <x:c r="B73" s="10"/>
+      <x:c r="C73" s="10"/>
       <x:c r="D73" s="9"/>
     </x:row>
     <x:row r="74">
-      <x:c r="A74" s="14"/>
-      <x:c r="B74" s="14"/>
-      <x:c r="C74" s="14"/>
+      <x:c r="A74" s="10"/>
+      <x:c r="B74" s="10"/>
+      <x:c r="C74" s="10"/>
       <x:c r="D74" s="9"/>
     </x:row>
     <x:row r="75">
-      <x:c r="A75" s="14"/>
-      <x:c r="B75" s="14"/>
-      <x:c r="C75" s="14"/>
+      <x:c r="A75" s="10"/>
+      <x:c r="B75" s="10"/>
+      <x:c r="C75" s="10"/>
       <x:c r="D75" s="9"/>
     </x:row>
     <x:row r="76">
-      <x:c r="A76" s="14"/>
-      <x:c r="B76" s="14"/>
-      <x:c r="C76" s="14"/>
+      <x:c r="A76" s="10"/>
+      <x:c r="B76" s="10"/>
+      <x:c r="C76" s="10"/>
       <x:c r="D76" s="9"/>
     </x:row>
     <x:row r="77">
-      <x:c r="A77" s="14"/>
-      <x:c r="B77" s="14"/>
-      <x:c r="C77" s="14"/>
+      <x:c r="A77" s="10"/>
+      <x:c r="B77" s="10"/>
+      <x:c r="C77" s="10"/>
       <x:c r="D77" s="9"/>
     </x:row>
     <x:row r="78">
-      <x:c r="A78" s="14"/>
-      <x:c r="B78" s="14"/>
-      <x:c r="C78" s="14"/>
+      <x:c r="A78" s="10"/>
+      <x:c r="B78" s="10"/>
+      <x:c r="C78" s="10"/>
       <x:c r="D78" s="9"/>
     </x:row>
     <x:row r="79">
-      <x:c r="A79" s="14"/>
-      <x:c r="B79" s="14"/>
-      <x:c r="C79" s="14"/>
+      <x:c r="A79" s="10"/>
+      <x:c r="B79" s="10"/>
+      <x:c r="C79" s="10"/>
       <x:c r="D79" s="9"/>
     </x:row>
     <x:row r="80">
-      <x:c r="A80" s="14"/>
-      <x:c r="B80" s="14"/>
-      <x:c r="C80" s="14"/>
+      <x:c r="A80" s="10"/>
+      <x:c r="B80" s="10"/>
+      <x:c r="C80" s="10"/>
       <x:c r="D80" s="9"/>
     </x:row>
     <x:row r="81">
-      <x:c r="A81" s="14"/>
-      <x:c r="B81" s="14"/>
-      <x:c r="C81" s="14"/>
+      <x:c r="A81" s="10"/>
+      <x:c r="B81" s="10"/>
+      <x:c r="C81" s="10"/>
       <x:c r="D81" s="9"/>
     </x:row>
     <x:row r="82">
-      <x:c r="A82" s="14"/>
-      <x:c r="B82" s="14"/>
-      <x:c r="C82" s="14"/>
+      <x:c r="A82" s="10"/>
+      <x:c r="B82" s="10"/>
+      <x:c r="C82" s="10"/>
       <x:c r="D82" s="9"/>
     </x:row>
     <x:row r="83">
-      <x:c r="A83" s="14"/>
-      <x:c r="B83" s="14"/>
-      <x:c r="C83" s="14"/>
+      <x:c r="A83" s="10"/>
+      <x:c r="B83" s="10"/>
+      <x:c r="C83" s="10"/>
       <x:c r="D83" s="9"/>
     </x:row>
     <x:row r="84">
-      <x:c r="A84" s="14"/>
-      <x:c r="B84" s="14"/>
-      <x:c r="C84" s="14"/>
+      <x:c r="A84" s="10"/>
+      <x:c r="B84" s="10"/>
+      <x:c r="C84" s="10"/>
       <x:c r="D84" s="9"/>
     </x:row>
     <x:row r="85">
-      <x:c r="A85" s="14"/>
-      <x:c r="B85" s="14"/>
-      <x:c r="C85" s="14"/>
+      <x:c r="A85" s="10"/>
+      <x:c r="B85" s="10"/>
+      <x:c r="C85" s="10"/>
       <x:c r="D85" s="9"/>
     </x:row>
     <x:row r="86">
-      <x:c r="A86" s="14"/>
-      <x:c r="B86" s="14"/>
-      <x:c r="C86" s="14"/>
+      <x:c r="A86" s="10"/>
+      <x:c r="B86" s="10"/>
+      <x:c r="C86" s="10"/>
       <x:c r="D86" s="9"/>
     </x:row>
     <x:row r="87">
-      <x:c r="A87" s="14"/>
-      <x:c r="B87" s="14"/>
-      <x:c r="C87" s="14"/>
+      <x:c r="A87" s="10"/>
+      <x:c r="B87" s="10"/>
+      <x:c r="C87" s="10"/>
       <x:c r="D87" s="9"/>
     </x:row>
     <x:row r="88">
-      <x:c r="A88" s="14"/>
-      <x:c r="B88" s="14"/>
-      <x:c r="C88" s="14"/>
+      <x:c r="A88" s="10"/>
+      <x:c r="B88" s="10"/>
+      <x:c r="C88" s="10"/>
       <x:c r="D88" s="9"/>
     </x:row>
     <x:row r="89">
-      <x:c r="A89" s="14"/>
-      <x:c r="B89" s="14"/>
-      <x:c r="C89" s="14"/>
+      <x:c r="A89" s="10"/>
+      <x:c r="B89" s="10"/>
+      <x:c r="C89" s="10"/>
       <x:c r="D89" s="9"/>
     </x:row>
     <x:row r="90">
-      <x:c r="A90" s="14"/>
-      <x:c r="B90" s="14"/>
-      <x:c r="C90" s="14"/>
+      <x:c r="A90" s="10"/>
+      <x:c r="B90" s="10"/>
+      <x:c r="C90" s="10"/>
       <x:c r="D90" s="9"/>
     </x:row>
     <x:row r="91">
-      <x:c r="A91" s="14"/>
-      <x:c r="B91" s="14"/>
-      <x:c r="C91" s="14"/>
+      <x:c r="A91" s="10"/>
+      <x:c r="B91" s="10"/>
+      <x:c r="C91" s="10"/>
       <x:c r="D91" s="9"/>
     </x:row>
     <x:row r="92">
-      <x:c r="A92" s="14"/>
-      <x:c r="B92" s="14"/>
-      <x:c r="C92" s="14"/>
+      <x:c r="A92" s="10"/>
+      <x:c r="B92" s="10"/>
+      <x:c r="C92" s="10"/>
       <x:c r="D92" s="9"/>
     </x:row>
     <x:row r="93">
-      <x:c r="A93" s="14"/>
-      <x:c r="B93" s="14"/>
-      <x:c r="C93" s="14"/>
+      <x:c r="A93" s="10"/>
+      <x:c r="B93" s="10"/>
+      <x:c r="C93" s="10"/>
       <x:c r="D93" s="9"/>
     </x:row>
     <x:row r="94">
-      <x:c r="A94" s="14"/>
-      <x:c r="B94" s="14"/>
-      <x:c r="C94" s="14"/>
+      <x:c r="A94" s="10"/>
+      <x:c r="B94" s="10"/>
+      <x:c r="C94" s="10"/>
       <x:c r="D94" s="9"/>
     </x:row>
     <x:row r="95">
-      <x:c r="A95" s="14"/>
-      <x:c r="B95" s="14"/>
-      <x:c r="C95" s="14"/>
+      <x:c r="A95" s="10"/>
+      <x:c r="B95" s="10"/>
+      <x:c r="C95" s="10"/>
       <x:c r="D95" s="9"/>
     </x:row>
     <x:row r="96">
-      <x:c r="A96" s="14"/>
-      <x:c r="B96" s="14"/>
-      <x:c r="C96" s="14"/>
+      <x:c r="A96" s="10"/>
+      <x:c r="B96" s="10"/>
+      <x:c r="C96" s="10"/>
       <x:c r="D96" s="9"/>
     </x:row>
     <x:row r="97">
-      <x:c r="A97" s="14"/>
-      <x:c r="B97" s="14"/>
-      <x:c r="C97" s="14"/>
+      <x:c r="A97" s="10"/>
+      <x:c r="B97" s="10"/>
+      <x:c r="C97" s="10"/>
       <x:c r="D97" s="9"/>
     </x:row>
     <x:row r="98">
-      <x:c r="A98" s="14"/>
-      <x:c r="B98" s="14"/>
-      <x:c r="C98" s="14"/>
+      <x:c r="A98" s="10"/>
+      <x:c r="B98" s="10"/>
+      <x:c r="C98" s="10"/>
       <x:c r="D98" s="9"/>
     </x:row>
     <x:row r="99">
-      <x:c r="A99" s="14"/>
-      <x:c r="B99" s="14"/>
-      <x:c r="C99" s="14"/>
+      <x:c r="A99" s="10"/>
+      <x:c r="B99" s="10"/>
+      <x:c r="C99" s="10"/>
       <x:c r="D99" s="9"/>
     </x:row>
     <x:row r="100">
-      <x:c r="A100" s="14"/>
-      <x:c r="B100" s="14"/>
-      <x:c r="C100" s="14"/>
+      <x:c r="A100" s="10"/>
+      <x:c r="B100" s="10"/>
+      <x:c r="C100" s="10"/>
       <x:c r="D100" s="9"/>
     </x:row>
     <x:row r="101">
-      <x:c r="A101" s="14"/>
-      <x:c r="B101" s="14"/>
-      <x:c r="C101" s="14"/>
+      <x:c r="A101" s="10"/>
+      <x:c r="B101" s="10"/>
+      <x:c r="C101" s="10"/>
       <x:c r="D101" s="9"/>
     </x:row>
   </x:sheetData>

</xml_diff>